<commit_message>
BLT: dùng logo thật, giữ tỉ lệ logo và tránh chữ đè logo
- Logo BLT Điện Nước thay logo tạm (cắt viền chụp màn hình, cắt sát nội dung)
- Ảnh logo neo một ô với kích thước theo đúng tỉ lệ thay vì kéo giãn
- Thu nhỏ chữ dòng địa chỉ/MST/email khi địa chỉ dài
- Cập nhật mẫu báo giá BLT

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Mau-bao-gia-BLT.xlsx
+++ b/bao-gia/BLT/Mau-bao-gia-BLT.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.##"/>
     <numFmt numFmtId="166" formatCode="#,##0;\-#,##0;\-"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -157,6 +157,13 @@
       <i val="1"/>
       <color rgb="FF7F7F7F"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <charset val="1"/>
+      <family val="0"/>
+      <color rgb="FF000000"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
   <fills count="6">
@@ -409,7 +416,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -599,46 +606,31 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
+  <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
-      <rowOff>0</rowOff>
+      <rowOff>19050</rowOff>
     </from>
-    <to>
-      <col>1</col>
-      <colOff>304200</colOff>
-      <row>3</row>
-      <rowOff>75600</rowOff>
-    </to>
+    <ext cx="952500" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="0" name="Image 1" descr="Picture"/>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="837720" cy="837720"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
-  </twoCellAnchor>
+  </oneCellAnchor>
 </wsDr>
 </file>
 

</xml_diff>